<commit_message>
Move plastics comparison out of part_tambahan.md into a Polikarbonat sheet in daftar_belanja.xlsx
- Removed the "Plastik Lain Selain Polikarbonat" subsection from
  part_tambahan.md (Sasis chapter reverts to just the main material table)
- Added a new "Polikarbonat" worksheet tab to daftar_belanja.xlsx covering
  polycarbonate plus the 5 alternatives (Delrin, HDPE, UHMW, Acrylic,
  Nylon), each with characteristics and a real Shopee link

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
+++ b/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Daftar Belanja" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Polikarbonat" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;US$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,6 +34,9 @@
     <font>
       <color rgb="FF0563C1"/>
       <u val="single"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -72,6 +76,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -544,4 +554,184 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Karakteristik</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Link Beli</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Polikarbonat (Lexan)</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Sangat tahan benturan, ringan, bisa transparan, mudah dipotong, harga terjangkau. Bukan buat struktur penahan beban utama.</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Polycarbonate-Sheet-3mm-Padat-Bening-Polikarbonat-Lembaran-Clear-i.358312392.3683120743</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Delrin / Acetal (POM)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Kuat, presisi tinggi, licin (low friction), relatif mahal. Cocok buat gear/bushing/motor mount.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/POM-Polyacetal-6mm-15x25cm-(Sheet-Lembaran)-Delrin-i.43613792.2387340703</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HDPE</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Relatif kuat, murah, ringan, tersedia lembaran relatif tipis. JANGAN dipotong laser (bisa terbakar).</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Nylon-PE-6mm-x-100cm-x-200cm-Lembaran-(-PolyEthylene-Sheet-HDPE-Plate-)-i.1247310023.49657775429</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>UHMW-PE</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Kuat, sangat tahan aus/gesekan, relatif mahal, biasanya lebih tebal. Cocok buat rail slide.</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/UHMWPE-12mm-100cm-x-200cm-Sheet-Lembaran-(-Polyethylene-)-i.43613792.9246365358</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Akrilik (Acrylic)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Murah, tersedia lembaran tipis (2-3mm), TAPI getas/rapuh - bukan struktural, cuma panel dekoratif/funnel.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Akrilik-Lembaran-Bening-3-mm-Acrylic-Sheet-Transparent-3mm-custom-laser-i.29403022.5739285630</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Nylon (PA6)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Kuat, tahan aus, relatif mahal, umumnya batangan (rod) bukan lembaran tipis - cocok buat poros/bushing.</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/nylon-rod-PA6-polyamide-110mm-engineering-plastic-resin-mc-cast-batang-i.418516762.21208902510</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Catatan: Nggak ada material di atas yang dilarang FTC. Aturan umum yang berlaku ke semua material: R202 (tidak boleh ada sisi tajam terekspos) dan R203 (tidak boleh material berbahaya kecuali disegel/dilapisi aman).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A9:D9"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Consolidate polycarbonate + alternatives into Sasis of part_minimum.md, add 2m purchase rows to spreadsheet
- part_minimum.md: Sasis now recommends a single popular polycarbonate
  thickness (3mm / 1/8in, the FTC standard per community sources) plus
  the 5 alternative plastics, each with a top Shopee/Tokopedia link
- part_tambahan.md: removed the 3 separate Polikarbonat rows and
  descriptive paragraph from the Sasis material table (now lives only
  in part_minimum.md); Rekomendasi updated to point there
- daftar_belanja.xlsx: added 6 rows to the Daftar Belanja sheet for 2m
  of each material (polycarbonate, Delrin, HDPE, UHMW, acrylic, nylon),
  with Total Harga formulas; extended the grand-total SUM range to H2:H8.
  Harga Satuan left blank for the new rows since Shopee blocks price
  scraping -- needs manual entry before the totals are meaningful

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
+++ b/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;US$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,10 @@
     </font>
     <font>
       <i val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -82,6 +86,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -537,20 +542,235 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Polikarbonat (Lexan) Sheet</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3mm, ~2m panjang (asumsi dijual per meter, cek satuan di listing)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Polycarbonate-Sheet-3mm-Padat-Bening-Polikarbonat-Lembaran-Clear-i.358312392.3683120743</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="2">
+        <f>E3*G3</f>
+        <v/>
+      </c>
+    </row>
     <row r="4">
-      <c r="G4" s="4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Delrin / Acetal (POM) Sheet</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>6mm, lembaran kecil (Delrin jarang dijual 2m - lihat catatan di part_minimum.md)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/POM-Polyacetal-6mm-15x25cm-(Sheet-Lembaran)-Delrin-i.43613792.2387340703</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="2">
+        <f>E4*G4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HDPE Sheet</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>6mm, 100cm x 200cm (1 lembar = 2m)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Nylon-PE-6mm-x-100cm-x-200cm-Lembaran-(-PolyEthylene-Sheet-HDPE-Plate-)-i.1247310023.49657775429</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2">
+        <f>E5*G5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UHMW-PE Sheet</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>12mm, 100cm x 200cm (1 lembar = 2m)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/UHMWPE-12mm-100cm-x-200cm-Sheet-Lembaran-(-Polyethylene-)-i.43613792.9246365358</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2">
+        <f>E6*G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Akrilik (Acrylic) Sheet</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>5mm, 100cm x 200cm (1 lembar = 2m)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/MIKA-AKRILIK-LEMBARAN-ACRYLIC-SHEET-5MM-X-100CM-X-200CM-i.1277418402.27123815875</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2">
+        <f>E7*G7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Nylon (PA6) Rod</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Dia. 25mm x 1m (butuh 2 batang buat 2m)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://shopee.co.id/Nylon-PA6-Putih-Batangan-(-PA6-Rod-White-)-Dia.-25-mm-x-1000-mm-i.68029486.1409073974</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="2">
+        <f>E8*G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="H4" s="5">
-        <f>SUM(H2:H2)</f>
+      <c r="H10" s="5">
+        <f>SUM(H2:H8)</f>
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Catatan: Harga Satuan material Sasis (baris 3-8) belum diisi - Shopee tidak bisa di-scrape harganya otomatis. Cek &amp; isi manual dari link sebelum checkout.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:H11"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Populate chassis material prices in daftar_belanja.xlsx, add USD<->IDR conversion
- Filled Harga Satuan (USD) for Polikarbonat, HDPE, UHMW, Akrilik, Nylon rod
  by converting real/reference IDR prices via a Kurs cell (K2), formula-linked
  so editing the rate recalculates every total automatically
- Added "Harga Asli (IDR)" column showing the source IDR price per row
- Added a second grand-total row "TOTAL KESELURUHAN (IDR)" right after the
  existing USD total, formula = USD total x kurs
- Delrin/Acetal left blank on purpose -- no reliable price found (Shopee/
  Tokopedia block scraping and it's not commonly sold in 2m sheets anyway);
  noted in the sheet to fill in manually
- Note: the Kurs cell is a manually-set reference rate (today's ~17,800),
  not a live auto-updating feed -- static xlsx files can't call external
  APIs; update the cell yourself when the rate moves and everything
  recalculates

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
+++ b/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
@@ -17,10 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;US$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;Rp&quot;#,##0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,10 @@
     </font>
     <font>
       <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -69,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -87,6 +92,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -463,6 +475,8 @@
     <col width="46" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,6 +520,16 @@
           <t>Total Harga</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Harga Asli (IDR)</t>
+        </is>
+      </c>
+      <c r="K1" s="9" t="inlineStr">
+        <is>
+          <t>Kurs USD -&gt; IDR (referensi 2026-08-20, update manual)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -541,6 +565,9 @@
         <f>E2*G2</f>
         <v/>
       </c>
+      <c r="K2" s="10" t="n">
+        <v>17800</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -561,7 +588,10 @@
           <t>3mm, ~2m panjang (asumsi dijual per meter, cek satuan di listing)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
+      <c r="E3" s="2">
+        <f>I3/$K$2</f>
+        <v/>
+      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>https://shopee.co.id/Polycarbonate-Sheet-3mm-Padat-Bening-Polikarbonat-Lembaran-Clear-i.358312392.3683120743</t>
@@ -573,6 +603,9 @@
       <c r="H3" s="2">
         <f>E3*G3</f>
         <v/>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>900000</v>
       </c>
     </row>
     <row r="4">
@@ -607,6 +640,11 @@
         <f>E4*G4</f>
         <v/>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Belum ketemu harga valid - cek manual</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -627,7 +665,10 @@
           <t>6mm, 100cm x 200cm (1 lembar = 2m)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n"/>
+      <c r="E5" s="2">
+        <f>I5/$K$2</f>
+        <v/>
+      </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>https://shopee.co.id/Nylon-PE-6mm-x-100cm-x-200cm-Lembaran-(-PolyEthylene-Sheet-HDPE-Plate-)-i.1247310023.49657775429</t>
@@ -639,6 +680,9 @@
       <c r="H5" s="2">
         <f>E5*G5</f>
         <v/>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>1300000</v>
       </c>
     </row>
     <row r="6">
@@ -660,7 +704,10 @@
           <t>12mm, 100cm x 200cm (1 lembar = 2m)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
+      <c r="E6" s="2">
+        <f>I6/$K$2</f>
+        <v/>
+      </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>https://shopee.co.id/UHMWPE-12mm-100cm-x-200cm-Sheet-Lembaran-(-Polyethylene-)-i.43613792.9246365358</t>
@@ -672,6 +719,9 @@
       <c r="H6" s="2">
         <f>E6*G6</f>
         <v/>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>1800000</v>
       </c>
     </row>
     <row r="7">
@@ -693,7 +743,10 @@
           <t>5mm, 100cm x 200cm (1 lembar = 2m)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n"/>
+      <c r="E7" s="2">
+        <f>I7/$K$2</f>
+        <v/>
+      </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
           <t>https://shopee.co.id/MIKA-AKRILIK-LEMBARAN-ACRYLIC-SHEET-5MM-X-100CM-X-200CM-i.1277418402.27123815875</t>
@@ -705,6 +758,9 @@
       <c r="H7" s="2">
         <f>E7*G7</f>
         <v/>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>313000</v>
       </c>
     </row>
     <row r="8">
@@ -726,7 +782,10 @@
           <t>Dia. 25mm x 1m (butuh 2 batang buat 2m)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="n"/>
+      <c r="E8" s="2">
+        <f>I8/$K$2</f>
+        <v/>
+      </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
           <t>https://shopee.co.id/Nylon-PA6-Putih-Batangan-(-PA6-Rod-White-)-Dia.-25-mm-x-1000-mm-i.68029486.1409073974</t>
@@ -739,8 +798,10 @@
         <f>E8*G8</f>
         <v/>
       </c>
-    </row>
-    <row r="9"/>
+      <c r="I8" s="11" t="n">
+        <v>70000</v>
+      </c>
+    </row>
     <row r="10">
       <c r="G10" s="4" t="inlineStr">
         <is>
@@ -753,15 +814,26 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Catatan: Harga Satuan material Sasis (baris 3-8) belum diisi - Shopee tidak bisa di-scrape harganya otomatis. Cek &amp; isi manual dari link sebelum checkout.</t>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL KESELURUHAN (IDR)</t>
+        </is>
+      </c>
+      <c r="H11" s="12">
+        <f>H10*$K$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Catatan harga: HDPE, Akrilik, Nylon rod = harga referensi dari listing Tokopedia/Indonetwork setara (bukan exact page Shopee, Shopee tidak bisa di-scrape). UHMW &amp; Polikarbonat = perkiraan/estimasi kasar (diskalakan dari data lain). Delrin = belum ketemu harga valid, kosong sengaja - isi manual dari link. Kurs IDR di K2 itu referensi manual (bukan live/auto-update) - update sendiri kalau kursnya sudah berubah, semua total bakal otomatis hitung ulang.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A12:I12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>

</xml_diff>

<commit_message>
Remove Delrin from Sasis material lists
- part_minimum.md: removed Delrin row from the Sasis table and its caveat note
- daftar_belanja.xlsx: removed Delrin from both the Daftar Belanja and
  Polikarbonat sheets, renumbered rows, fixed formula references and the
  SUM range that delete_rows left stale, cleaned up stray merged-cell/
  hyperlink artifacts left over from the row deletion

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
+++ b/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
@@ -619,31 +619,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Delrin / Acetal (POM) Sheet</t>
+          <t>HDPE Sheet</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6mm, lembaran kecil (Delrin jarang dijual 2m - lihat catatan di part_minimum.md)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n"/>
+          <t>6mm, 100cm x 200cm (1 lembar = 2m)</t>
+        </is>
+      </c>
+      <c r="E4" s="2">
+        <f>I4/$K$2</f>
+        <v/>
+      </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/POM-Polyacetal-6mm-15x25cm-(Sheet-Lembaran)-Delrin-i.43613792.2387340703</t>
+          <t>https://shopee.co.id/Nylon-PE-6mm-x-100cm-x-200cm-Lembaran-(-PolyEthylene-Sheet-HDPE-Plate-)-i.1247310023.49657775429</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" s="2">
         <f>E4*G4</f>
         <v/>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Belum ketemu harga valid - cek manual</t>
-        </is>
+      <c r="I4" s="11" t="n">
+        <v>1300000</v>
       </c>
     </row>
     <row r="5">
@@ -657,12 +658,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>HDPE Sheet</t>
+          <t>UHMW-PE Sheet</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6mm, 100cm x 200cm (1 lembar = 2m)</t>
+          <t>12mm, 100cm x 200cm (1 lembar = 2m)</t>
         </is>
       </c>
       <c r="E5" s="2">
@@ -671,7 +672,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/Nylon-PE-6mm-x-100cm-x-200cm-Lembaran-(-PolyEthylene-Sheet-HDPE-Plate-)-i.1247310023.49657775429</t>
+          <t>https://shopee.co.id/UHMWPE-12mm-100cm-x-200cm-Sheet-Lembaran-(-Polyethylene-)-i.43613792.9246365358</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -682,7 +683,7 @@
         <v/>
       </c>
       <c r="I5" s="11" t="n">
-        <v>1300000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="6">
@@ -696,12 +697,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>UHMW-PE Sheet</t>
+          <t>Akrilik (Acrylic) Sheet</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>12mm, 100cm x 200cm (1 lembar = 2m)</t>
+          <t>5mm, 100cm x 200cm (1 lembar = 2m)</t>
         </is>
       </c>
       <c r="E6" s="2">
@@ -710,7 +711,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/UHMWPE-12mm-100cm-x-200cm-Sheet-Lembaran-(-Polyethylene-)-i.43613792.9246365358</t>
+          <t>https://shopee.co.id/MIKA-AKRILIK-LEMBARAN-ACRYLIC-SHEET-5MM-X-100CM-X-200CM-i.1277418402.27123815875</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -721,7 +722,7 @@
         <v/>
       </c>
       <c r="I6" s="11" t="n">
-        <v>1800000</v>
+        <v>313000</v>
       </c>
     </row>
     <row r="7">
@@ -735,12 +736,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Akrilik (Acrylic) Sheet</t>
+          <t>Nylon (PA6) Rod</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5mm, 100cm x 200cm (1 lembar = 2m)</t>
+          <t>Dia. 25mm x 1m (butuh 2 batang buat 2m)</t>
         </is>
       </c>
       <c r="E7" s="2">
@@ -749,88 +750,50 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/MIKA-AKRILIK-LEMBARAN-ACRYLIC-SHEET-5MM-X-100CM-X-200CM-i.1277418402.27123815875</t>
+          <t>https://shopee.co.id/Nylon-PA6-Putih-Batangan-(-PA6-Rod-White-)-Dia.-25-mm-x-1000-mm-i.68029486.1409073974</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" s="2">
         <f>E7*G7</f>
         <v/>
       </c>
       <c r="I7" s="11" t="n">
-        <v>313000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Nylon (PA6) Rod</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Dia. 25mm x 1m (butuh 2 batang buat 2m)</t>
-        </is>
-      </c>
-      <c r="E8" s="2">
-        <f>I8/$K$2</f>
-        <v/>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>https://shopee.co.id/Nylon-PA6-Putih-Batangan-(-PA6-Rod-White-)-Dia.-25-mm-x-1000-mm-i.68029486.1409073974</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="2">
-        <f>E8*G8</f>
-        <v/>
-      </c>
-      <c r="I8" s="11" t="n">
         <v>70000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL KESELURUHAN</t>
+        </is>
+      </c>
+      <c r="H9" s="5">
+        <f>SUM(H2:H7)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>TOTAL KESELURUHAN</t>
-        </is>
-      </c>
-      <c r="H10" s="5">
-        <f>SUM(H2:H8)</f>
+          <t>TOTAL KESELURUHAN (IDR)</t>
+        </is>
+      </c>
+      <c r="H10" s="12">
+        <f>H9*$K$2</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL KESELURUHAN (IDR)</t>
-        </is>
-      </c>
-      <c r="H11" s="12">
-        <f>H10*$K$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Catatan harga: HDPE, Akrilik, Nylon rod = harga referensi dari listing Tokopedia/Indonetwork setara (bukan exact page Shopee, Shopee tidak bisa di-scrape). UHMW &amp; Polikarbonat = perkiraan/estimasi kasar (diskalakan dari data lain). Delrin = belum ketemu harga valid, kosong sengaja - isi manual dari link. Kurs IDR di K2 itu referensi manual (bukan live/auto-update) - update sendiri kalau kursnya sudah berubah, semua total bakal otomatis hitung ulang.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Catatan harga: HDPE, Akrilik, Nylon rod = harga referensi dari listing Tokopedia/Indonetwork setara (bukan exact page Shopee, Shopee tidak bisa di-scrape). UHMW &amp; Polikarbonat = perkiraan/estimasi kasar (diskalakan dari data lain). Kurs IDR di K2 itu referensi manual (bukan live/auto-update) - update sendiri kalau kursnya sudah berubah, semua total bakal otomatis hitung ulang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A12:I12"/>
@@ -838,11 +801,9 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -854,7 +815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -911,17 +872,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Delrin / Acetal (POM)</t>
+          <t>HDPE</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Kuat, presisi tinggi, licin (low friction), relatif mahal. Cocok buat gear/bushing/motor mount.</t>
+          <t>Relatif kuat, murah, ringan, tersedia lembaran relatif tipis. JANGAN dipotong laser (bisa terbakar).</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/POM-Polyacetal-6mm-15x25cm-(Sheet-Lembaran)-Delrin-i.43613792.2387340703</t>
+          <t>https://shopee.co.id/Nylon-PE-6mm-x-100cm-x-200cm-Lembaran-(-PolyEthylene-Sheet-HDPE-Plate-)-i.1247310023.49657775429</t>
         </is>
       </c>
     </row>
@@ -931,17 +892,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HDPE</t>
+          <t>UHMW-PE</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Relatif kuat, murah, ringan, tersedia lembaran relatif tipis. JANGAN dipotong laser (bisa terbakar).</t>
+          <t>Kuat, sangat tahan aus/gesekan, relatif mahal, biasanya lebih tebal. Cocok buat rail slide.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/Nylon-PE-6mm-x-100cm-x-200cm-Lembaran-(-PolyEthylene-Sheet-HDPE-Plate-)-i.1247310023.49657775429</t>
+          <t>https://shopee.co.id/UHMWPE-12mm-100cm-x-200cm-Sheet-Lembaran-(-Polyethylene-)-i.43613792.9246365358</t>
         </is>
       </c>
     </row>
@@ -951,17 +912,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UHMW-PE</t>
+          <t>Akrilik (Acrylic)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Kuat, sangat tahan aus/gesekan, relatif mahal, biasanya lebih tebal. Cocok buat rail slide.</t>
+          <t>Murah, tersedia lembaran tipis (2-3mm), TAPI getas/rapuh - bukan struktural, cuma panel dekoratif/funnel.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/UHMWPE-12mm-100cm-x-200cm-Sheet-Lembaran-(-Polyethylene-)-i.43613792.9246365358</t>
+          <t>https://shopee.co.id/Akrilik-Lembaran-Bening-3-mm-Acrylic-Sheet-Transparent-3mm-custom-laser-i.29403022.5739285630</t>
         </is>
       </c>
     </row>
@@ -971,42 +932,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Akrilik (Acrylic)</t>
+          <t>Nylon (PA6)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Murah, tersedia lembaran tipis (2-3mm), TAPI getas/rapuh - bukan struktural, cuma panel dekoratif/funnel.</t>
+          <t>Kuat, tahan aus, relatif mahal, umumnya batangan (rod) bukan lembaran tipis - cocok buat poros/bushing.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>https://shopee.co.id/Akrilik-Lembaran-Bening-3-mm-Acrylic-Sheet-Transparent-3mm-custom-laser-i.29403022.5739285630</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Nylon (PA6)</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Kuat, tahan aus, relatif mahal, umumnya batangan (rod) bukan lembaran tipis - cocok buat poros/bushing.</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
           <t>https://shopee.co.id/nylon-rod-PA6-polyamide-110mm-engineering-plastic-resin-mc-cast-batang-i.418516762.21208902510</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="7" ht="30" customHeight="1"/>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Catatan: Nggak ada material di atas yang dilarang FTC. Aturan umum yang berlaku ke semua material: R202 (tidak boleh ada sisi tajam terekspos) dan R203 (tidak boleh material berbahaya kecuali disegel/dilapisi aman).</t>
         </is>
@@ -1014,15 +956,13 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A8:D8"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Pengambil and Pelontar in part_minimum.md, add Pelontar motor row to spreadsheet
- Pengambil: clarified as 2x Core Hex Motor owned (1 per bot), fully covers
  both robots' intake, 0 dibeli
- Pelontar: now requires 4x HD Hex Motor (2 per bot x 2 bots), all bought
  fresh since the 6 owned are already committed to Penggerak/drivetrain
- daftar_belanja.xlsx: added the 4x HD Hex Motor Pelontar row, fixed the
  SUM range and IDR-total formula reference after the insert (verified
  row-by-row to avoid repeating the earlier insert_rows formula-shift bug)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
+++ b/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
@@ -764,36 +764,70 @@
         <v>70000</v>
       </c>
     </row>
-    <row r="9">
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL KESELURUHAN</t>
-        </is>
-      </c>
-      <c r="H9" s="5">
-        <f>SUM(H2:H7)</f>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>REV-41-1600</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UltraPlanetary Gearbox Kit &amp; HD Hex Motor</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>HD Hex Motor (buat Pelontar, 2 per bot x 2 bot)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.revrobotics.com/rev-41-1600/</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="2">
+        <f>E8*G8</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="G10" s="4" t="inlineStr">
         <is>
+          <t>TOTAL KESELURUHAN</t>
+        </is>
+      </c>
+      <c r="H10" s="5">
+        <f>SUM(H2:H8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="G11" s="4" t="inlineStr">
+        <is>
           <t>TOTAL KESELURUHAN (IDR)</t>
         </is>
       </c>
-      <c r="H10" s="12">
-        <f>H9*$K$2</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="H11" s="12">
+        <f>H10*$K$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Catatan harga: HDPE, Akrilik, Nylon rod = harga referensi dari listing Tokopedia/Indonetwork setara (bukan exact page Shopee, Shopee tidak bisa di-scrape). UHMW &amp; Polikarbonat = perkiraan/estimasi kasar (diskalakan dari data lain). Kurs IDR di K2 itu referensi manual (bukan live/auto-update) - update sendiri kalau kursnya sudah berubah, semua total bakal otomatis hitung ulang.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A12:I12"/>
@@ -804,6 +838,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge duplicate HD Hex Motor rows into one, remove Catatan Harga note
- Combined the two separate REV-41-1600 rows (2 for Penggerak, 4 for
  Pelontar) into a single row with qty 6, description covering both uses
- Removed the Catatan Harga note row entirely
- Rebuilt the sheet from scratch (clearing and rewriting all rows) rather
  than incremental insert/delete, to avoid repeating the formula-reference
  bug from earlier edits

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
+++ b/parts/Part yang Perlu Dibeli/daftar_belanja.xlsx
@@ -74,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -99,6 +99,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -547,7 +548,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>HD Hex Motor</t>
+          <t>HD Hex Motor (2 buat Penggerak + 4 buat Pelontar)</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -559,7 +560,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H2" s="2">
         <f>E2*G2</f>
@@ -765,80 +766,48 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>REV-41-1600</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>UltraPlanetary Gearbox Kit &amp; HD Hex Motor</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>HD Hex Motor (buat Pelontar, 2 per bot x 2 bot)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>https://www.revrobotics.com/rev-41-1600/</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>4</v>
-      </c>
-      <c r="H8" s="2">
-        <f>E8*G8</f>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="H8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL KESELURUHAN</t>
+        </is>
+      </c>
+      <c r="H9" s="5">
+        <f>SUM(H2:H7)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>TOTAL KESELURUHAN</t>
-        </is>
-      </c>
-      <c r="H10" s="5">
-        <f>SUM(H2:H8)</f>
+          <t>TOTAL KESELURUHAN (IDR)</t>
+        </is>
+      </c>
+      <c r="H10" s="12">
+        <f>H9*$K$2</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL KESELURUHAN (IDR)</t>
-        </is>
-      </c>
-      <c r="H11" s="12">
-        <f>H10*$K$2</f>
-        <v/>
-      </c>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="12" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Catatan harga: HDPE, Akrilik, Nylon rod = harga referensi dari listing Tokopedia/Indonetwork setara (bukan exact page Shopee, Shopee tidak bisa di-scrape). UHMW &amp; Polikarbonat = perkiraan/estimasi kasar (diskalakan dari data lain). Kurs IDR di K2 itu referensi manual (bukan live/auto-update) - update sendiri kalau kursnya sudah berubah, semua total bakal otomatis hitung ulang.</t>
-        </is>
-      </c>
-    </row>
+      <c r="A12" s="13" t="n"/>
+    </row>
+    <row r="13"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A12:I12"/>
-  </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>